<commit_message>
Improved and debug API requests
</commit_message>
<xml_diff>
--- a/setup_files/all_raw_materials.xlsx
+++ b/setup_files/all_raw_materials.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\MBPI-Projects\RM-Consumption-Management-System-Backend-API\setup_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\MBPI-Projects\DEPLOYMENT-WAREHOUSE-PROGRAM-BACKEND\setup_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E56E2E7-73FA-497E-9BDA-62616F6AB806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBD0FC8B-A556-47E9-852B-A75A931874CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F20E24F6-91ED-4D57-ADFF-F15466AAF156}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="314">
   <si>
     <t>rm_code</t>
   </si>
@@ -922,13 +922,58 @@
   </si>
   <si>
     <t xml:space="preserve">Y89 </t>
+  </si>
+  <si>
+    <t>SAMPLE 1</t>
+  </si>
+  <si>
+    <t>SAMPLE 2</t>
+  </si>
+  <si>
+    <t>SAMPLE 3</t>
+  </si>
+  <si>
+    <t>SAMPLE 4</t>
+  </si>
+  <si>
+    <t>SAMPLE 5</t>
+  </si>
+  <si>
+    <t>SAMPLE 6</t>
+  </si>
+  <si>
+    <t>SAMPLE 7</t>
+  </si>
+  <si>
+    <t>SAMPLE 8</t>
+  </si>
+  <si>
+    <t>SAMPLE 9</t>
+  </si>
+  <si>
+    <t>SAMPLE 10</t>
+  </si>
+  <si>
+    <t>SAMPLE 11</t>
+  </si>
+  <si>
+    <t>SAMPLE 12</t>
+  </si>
+  <si>
+    <t>SAMPLE 13</t>
+  </si>
+  <si>
+    <t>SAMPLE 14</t>
+  </si>
+  <si>
+    <t>SAMPLE 15</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -951,6 +996,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -960,7 +1011,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -983,11 +1034,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -999,6 +1061,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1315,7 +1380,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA8A97F4-DB29-4550-9F6D-3DE503E71245}">
-  <dimension ref="A1:A299"/>
+  <dimension ref="A1:A314"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
@@ -2816,7 +2881,83 @@
         <v>274</v>
       </c>
     </row>
+    <row r="300" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A300" s="5" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="301" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A301" s="5" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="302" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A302" s="5" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="303" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A303" s="5" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="304" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A304" s="5" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="305" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A305" s="5" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="306" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A306" s="5" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="307" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A307" s="5" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="308" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A308" s="5" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="309" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A309" s="5" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="310" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A310" s="5" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="311" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A311" s="5" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="312" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A312" s="5" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="313" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A313" s="5" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="314" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A314" s="5" t="s">
+        <v>313</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>